<commit_message>
fix(import_pracownikow): utwardzenie pliku wzorcowego wg self-review Codeksa
- dane przykladowe oczywiscie testowe (Przykladowy/Testowy, jednostka
  "Przykladowa Katedra Testowa", bez realistycznego ORCID) — kto zapomni
  skasowac wierszy przykladowych, nie zaimportuje realnie brzmiacych osob
  ani nie trafi po identyfikatorze w istniejacy rekord;
- komenda generuj_plik_wzorcowy odmawia zapisu przez symlink (CommandError)
  — chroni tests/testdata.xlsx przy regeneracji na starym checkoutcie;
- test: plik wzorcowy jest faktycznie XLSX (wykryj_format), nie CSV udajacy
  xlsx po rozszerzeniu; test regresyjny guardu symlinku;
- doc: link "plik wzorcowy na GitHub" wskazuje na plik wzorcowy static,
  nie surowy fixture tests/testdata.xlsx.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/import_pracownikow/static/import_pracownikow/import_pracownikow_przyklad.xlsx
+++ b/src/import_pracownikow/static/import_pracownikow/import_pracownikow_przyklad.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Kowalski</t>
+          <t>Przykładowy</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -569,12 +569,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Katedra i Klinika Dermatologii</t>
+          <t>Przykładowa Katedra Testowa</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Wydział Lekarski</t>
+          <t>Przykładowy Wydział</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -599,7 +599,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Nowak</t>
+          <t>Przykładowa</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -607,11 +607,6 @@
           <t>Maria</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>0000-0002-2752-5144</t>
-        </is>
-      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>dr n. med.</t>
@@ -629,12 +624,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Katedra Testowa</t>
+          <t>Przykładowa Katedra Testowa</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Wydział Lekarski</t>
+          <t>Przykładowy Wydział</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -659,7 +654,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Wiśniewski</t>
+          <t>Testowy</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -684,12 +679,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Katedra Testowa</t>
+          <t>Przykładowa Katedra Testowa</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Wydział Lekarski</t>
+          <t>Przykładowy Wydział</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -716,7 +711,7 @@
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t>Lubelska</t>
+          <t>Testowa</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -726,7 +721,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Katedra Testowa</t>
+          <t>Przykładowa Katedra Testowa</t>
         </is>
       </c>
     </row>

</xml_diff>